<commit_message>
Improve image search reliability and UI
</commit_message>
<xml_diff>
--- a/data/processing_report.xlsx
+++ b/data/processing_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N212"/>
+  <dimension ref="A1:O212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -437,12 +437,13 @@
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="48" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="50" customWidth="1" min="11" max="11"/>
     <col width="50" customWidth="1" min="12" max="12"/>
     <col width="19" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -514,6 +515,11 @@
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Dimensions</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Drive Link</t>
         </is>
       </c>
     </row>
@@ -550,12 +556,13 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests (015d12c) for url: https://upload.wikimedia.org/wikipedia/commons/d/d2/Grilled_Tandoori_chicken.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
+          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/d/d2/Grilled_Tandoori_chicken.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -590,12 +597,13 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests (015d12c) for url: https://upload.wikimedia.org/wikipedia/commons/a/a7/Veg_Fried_Rice_%2851465%29.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
+          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/a/a7/Veg_Fried_Rice_%2851465%29.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -618,7 +626,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -643,14 +651,10 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>&lt;HttpError 404 when requesting None returned "File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.". Details: "[{'message': 'File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.', 'domain': 'global', 'reason': 'notFound', 'location': 'fileId', 'locationType': 'parameter'}]"&gt;</t>
-        </is>
-      </c>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Chicken Biryani Boneless.jpg</t>
@@ -664,6 +668,11 @@
           <t>1800x1200</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1t_jEAFC5X9VnVXg_1qlATI1DU3n-8aNA/view?usp=drivesdk</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -676,12 +685,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>84</v>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -689,26 +696,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Wikimedia Commons</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/?curid=87676537</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>CC BY-SA 4.0</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>User:Oganguly</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>Failed</t>
@@ -716,22 +707,13 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>&lt;HttpError 404 when requesting None returned "File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.". Details: "[{'message': 'File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.', 'domain': 'global', 'reason': 'notFound', 'location': 'fileId', 'locationType': 'parameter'}]"&gt;</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Butter Roti.jpg</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>681781</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>1800x1200</t>
-        </is>
-      </c>
+          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/4/4b/Hamburger_America_peanut_butter_and_jelly.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -754,7 +736,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -779,14 +761,10 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>&lt;HttpError 404 when requesting None returned "File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.". Details: "[{'message': 'File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.', 'domain': 'global', 'reason': 'notFound', 'location': 'fileId', 'locationType': 'parameter'}]"&gt;</t>
-        </is>
-      </c>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Paneer Tikka Masala.jpg</t>
@@ -800,6 +778,11 @@
           <t>1800x1200</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1FWTodjAdW4AYA-eiUHLslj_ilKu66Nhv/view?usp=drivesdk</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -822,7 +805,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -847,14 +830,10 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>&lt;HttpError 404 when requesting None returned "File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.". Details: "[{'message': 'File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.', 'domain': 'global', 'reason': 'notFound', 'location': 'fileId', 'locationType': 'parameter'}]"&gt;</t>
-        </is>
-      </c>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Chicken Fried Rice.jpg</t>
@@ -866,6 +845,11 @@
       <c r="N7" t="inlineStr">
         <is>
           <t>1800x1200</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1rApKulJ4DdmDXDS0Uc5rPab_tmXvhCfP/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -908,6 +892,7 @@
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -930,7 +915,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -955,14 +940,10 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>&lt;HttpError 404 when requesting None returned "File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.". Details: "[{'message': 'File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.', 'domain': 'global', 'reason': 'notFound', 'location': 'fileId', 'locationType': 'parameter'}]"&gt;</t>
-        </is>
-      </c>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Roti.jpg</t>
@@ -976,6 +957,11 @@
           <t>1800x1200</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/16XSc9ZDUiY6wz3IGkmZVLWjN5CkXjp3e/view?usp=drivesdk</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -998,7 +984,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1023,14 +1009,10 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>&lt;HttpError 404 when requesting None returned "File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.". Details: "[{'message': 'File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.', 'domain': 'global', 'reason': 'notFound', 'location': 'fileId', 'locationType': 'parameter'}]"&gt;</t>
-        </is>
-      </c>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Chicken Tandoori [Half].jpg</t>
@@ -1042,6 +1024,11 @@
       <c r="N10" t="inlineStr">
         <is>
           <t>1800x1200</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1rvV7WpsjwrPDLe6WNxahQgA7k_khMq7e/view?usp=drivesdk</t>
         </is>
       </c>
     </row>
@@ -1084,6 +1071,7 @@
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1124,6 +1112,7 @@
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1164,6 +1153,7 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1204,6 +1194,7 @@
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1213,15 +1204,13 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>100</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1229,26 +1218,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Wikimedia Commons</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/?curid=103959326</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>CC BY-SA 4.0</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>G.HarishGovindaraj</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>Failed</t>
@@ -1256,22 +1229,13 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>&lt;HttpError 404 when requesting None returned "File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.". Details: "[{'message': 'File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.', 'domain': 'global', 'reason': 'notFound', 'location': 'fileId', 'locationType': 'parameter'}]"&gt;</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Chicken Chilli.jpg</t>
-        </is>
-      </c>
-      <c r="M15" t="n">
-        <v>470247</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>1800x1200</t>
-        </is>
-      </c>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Chilli&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1281,15 +1245,13 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>100</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1297,27 +1259,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Wikimedia Commons</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/?curid=157375737</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>CC BY-SA 4.0</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Author: Karel Frederik Holle (1894, 1904/1911, 1931), Stokhof, W.A.L. editor (1980-1987)
-Journal: Pacific Linguistics</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
           <t>Failed</t>
@@ -1325,22 +1270,13 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>&lt;HttpError 404 when requesting None returned "File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.". Details: "[{'message': 'File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.', 'domain': 'global', 'reason': 'notFound', 'location': 'fileId', 'locationType': 'parameter'}]"&gt;</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Chicken Kala Masala.jpg</t>
-        </is>
-      </c>
-      <c r="M16" t="n">
-        <v>131761</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>1800x1200</t>
-        </is>
-      </c>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Kala+Masala&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1350,15 +1286,13 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>75</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1366,26 +1300,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Wikimedia Commons</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/?curid=102245001</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>CC BY-SA 4.0</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>AugustineKajur</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>Failed</t>
@@ -1393,22 +1311,13 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>&lt;HttpError 404 when requesting None returned "File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.". Details: "[{'message': 'File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.', 'domain': 'global', 'reason': 'notFound', 'location': 'fileId', 'locationType': 'parameter'}]"&gt;</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Dal Tadka.jpg</t>
-        </is>
-      </c>
-      <c r="M17" t="n">
-        <v>477712</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>1800x1200</t>
-        </is>
-      </c>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Dal+Tadka&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1418,15 +1327,13 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>100</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1434,26 +1341,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Wikimedia Commons</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/?curid=103141752</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>CC BY-SA 4.0</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Vipul7229</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
           <t>Failed</t>
@@ -1461,22 +1352,13 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>&lt;HttpError 404 when requesting None returned "File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.". Details: "[{'message': 'File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.', 'domain': 'global', 'reason': 'notFound', 'location': 'fileId', 'locationType': 'parameter'}]"&gt;</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Paneer Crispy.jpg</t>
-        </is>
-      </c>
-      <c r="M18" t="n">
-        <v>782170</v>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>1800x1200</t>
-        </is>
-      </c>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Paneer+Crispy&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1486,7 +1368,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -1511,12 +1393,13 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests (015d12c) for url: https://upload.wikimedia.org/wikipedia/commons/2/29/Butter_Naan_2.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Butter+Naan&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1526,15 +1409,13 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>100</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1542,26 +1423,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Wikimedia Commons</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/?curid=190429834</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>CC BY-SA 4.0</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Bahnfrend</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
           <t>Failed</t>
@@ -1569,22 +1434,13 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>&lt;HttpError 404 when requesting None returned "File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.". Details: "[{'message': 'File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.', 'domain': 'global', 'reason': 'notFound', 'location': 'fileId', 'locationType': 'parameter'}]"&gt;</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Chicken Crispy.jpg</t>
-        </is>
-      </c>
-      <c r="M20" t="n">
-        <v>534616</v>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>1800x1200</t>
-        </is>
-      </c>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Crispy&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1594,7 +1450,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1619,12 +1475,13 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests (015d12c) for url: https://upload.wikimedia.org/wikipedia/commons/9/9b/Chicken_Gravy_%22Jhol%22.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Masala+Boneless&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1634,15 +1491,13 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>83</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1650,26 +1505,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Wikimedia Commons</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>https://commons.wikimedia.org/?curid=103645608</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>CC BY-SA 4.0</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Souradeep Roy 1998</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>Failed</t>
@@ -1677,22 +1516,13 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>&lt;HttpError 404 when requesting None returned "File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.". Details: "[{'message': 'File not found: https://drive.google.com/drive/folders/1vhfw2VtIb0jclNeNKslHjhrC4dpYWVHd.', 'domain': 'global', 'reason': 'notFound', 'location': 'fileId', 'locationType': 'parameter'}]"&gt;</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Chicken Tandoori (Half).jpg</t>
-        </is>
-      </c>
-      <c r="M22" t="n">
-        <v>527563</v>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>1800x1200</t>
-        </is>
-      </c>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Tandoori+%28Half%29&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1702,7 +1532,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1727,12 +1557,13 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>All candidate images failed basic quality checks.</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Veg+Handi&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1742,7 +1573,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1767,12 +1598,13 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/8/84/Dum_veg_biryani_by_fatima.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Veg+Dum+Biryani&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1813,6 +1645,7 @@
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1853,6 +1686,7 @@
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1893,6 +1727,7 @@
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1933,6 +1768,7 @@
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1973,6 +1809,7 @@
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2013,6 +1850,7 @@
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2053,6 +1891,7 @@
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2093,6 +1932,7 @@
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2133,6 +1973,7 @@
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2173,6 +2014,7 @@
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2213,6 +2055,7 @@
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2253,6 +2096,7 @@
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2293,6 +2137,7 @@
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2333,6 +2178,7 @@
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2373,6 +2219,7 @@
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2413,6 +2260,7 @@
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2453,6 +2301,7 @@
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2493,6 +2342,7 @@
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2533,6 +2383,7 @@
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2573,6 +2424,7 @@
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2613,6 +2465,7 @@
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2653,6 +2506,7 @@
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2693,6 +2547,7 @@
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2733,6 +2588,7 @@
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2773,6 +2629,7 @@
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2813,6 +2670,7 @@
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2853,6 +2711,7 @@
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2893,6 +2752,7 @@
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2933,6 +2793,7 @@
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2973,6 +2834,7 @@
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3013,6 +2875,7 @@
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3053,6 +2916,7 @@
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3093,6 +2957,7 @@
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3133,6 +2998,7 @@
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3173,6 +3039,7 @@
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3182,37 +3049,66 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>91</v>
+      </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/?curid=131505199</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>CC BY 3.0</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Biswarup Ganguly</t>
+        </is>
+      </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Hot+Garlic&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Chicken Hot Garlic.jpg</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>488151</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>1800x1200</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1PdCIOvj_Zan0dCDFUexLSyW3mqK6BVxv/view?usp=drivesdk</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3222,7 +3118,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
@@ -3247,12 +3143,13 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Veg+Hyderabadi+Biryani&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/7/7f/Hyderabadi_Veg_Biryani.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
         </is>
       </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3262,7 +3159,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
@@ -3287,12 +3184,13 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Veg+Kadai&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/f/fc/Kadai_Paneer_Recipe.JPG?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
         </is>
       </c>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3302,37 +3200,66 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>100</v>
+      </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/?curid=40984113</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Kajori.p</t>
+        </is>
+      </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Mutton+Rogan+Josh&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Mutton Rogan Josh.jpg</t>
+        </is>
+      </c>
+      <c r="M63" t="n">
+        <v>515731</v>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>1800x1200</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1YuC7RUNyvRrzw6ZdARHPsGkGYtafKS1I/view?usp=drivesdk</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3367,12 +3294,13 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Veg+Schezwan+Fried+Rice&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Veg+Schezwan+Fried+Rice+dish&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3413,6 +3341,7 @@
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3453,6 +3382,7 @@
       <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3493,6 +3423,7 @@
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3533,6 +3464,7 @@
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3573,6 +3505,7 @@
       <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3613,6 +3546,7 @@
       <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3653,6 +3587,7 @@
       <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3693,6 +3628,7 @@
       <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3733,6 +3669,7 @@
       <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr"/>
       <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3742,7 +3679,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -3767,12 +3704,13 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/c/cb/Fries_%2814918258342%29.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Fingers+Chips&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr"/>
       <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3807,12 +3745,13 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>No image candidates found.</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Veg+Diwani+Handi&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr"/>
       <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3822,7 +3761,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -3847,12 +3786,13 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/b/b0/Chicken_Manchow_Soup.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Manchow+Soup&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3887,12 +3827,13 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>No image candidates found.</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Mushroom+Tikka+Biryani&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3927,12 +3868,13 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Manchurian+Fried+Rice+dish&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Manchurian+Fried+Rice&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3973,6 +3915,7 @@
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4013,6 +3956,7 @@
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4053,6 +3997,7 @@
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4093,6 +4038,7 @@
       <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr"/>
       <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4133,6 +4079,7 @@
       <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4173,6 +4120,7 @@
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr"/>
       <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4213,6 +4161,7 @@
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr"/>
       <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4253,6 +4202,7 @@
       <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4293,6 +4243,7 @@
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr"/>
       <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4333,6 +4284,7 @@
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4373,6 +4325,7 @@
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr"/>
       <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4413,6 +4366,7 @@
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr"/>
       <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4453,6 +4407,7 @@
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4493,6 +4448,7 @@
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr"/>
       <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4533,6 +4489,7 @@
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr"/>
       <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4573,6 +4530,7 @@
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4613,6 +4571,7 @@
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4653,6 +4612,7 @@
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr"/>
       <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4693,6 +4653,7 @@
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr"/>
       <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4733,6 +4694,7 @@
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr"/>
       <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4773,6 +4735,7 @@
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr"/>
       <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4813,6 +4776,7 @@
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr"/>
+      <c r="O100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4853,6 +4817,7 @@
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr"/>
       <c r="N101" t="inlineStr"/>
+      <c r="O101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4893,6 +4858,7 @@
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr"/>
       <c r="N102" t="inlineStr"/>
+      <c r="O102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4933,6 +4899,7 @@
       <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr"/>
       <c r="N103" t="inlineStr"/>
+      <c r="O103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4973,6 +4940,7 @@
       <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr"/>
       <c r="N104" t="inlineStr"/>
+      <c r="O104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5013,6 +4981,7 @@
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr"/>
       <c r="N105" t="inlineStr"/>
+      <c r="O105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5053,6 +5022,7 @@
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr"/>
       <c r="N106" t="inlineStr"/>
+      <c r="O106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5093,6 +5063,7 @@
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr"/>
       <c r="N107" t="inlineStr"/>
+      <c r="O107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5133,6 +5104,7 @@
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr"/>
       <c r="N108" t="inlineStr"/>
+      <c r="O108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5173,6 +5145,7 @@
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr"/>
       <c r="N109" t="inlineStr"/>
+      <c r="O109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5182,7 +5155,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C110" t="inlineStr"/>
@@ -5207,12 +5180,13 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Veg+Combination+Fried+Rice&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+          <t>No candidate met AI threshold 75; best score 71.</t>
         </is>
       </c>
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr"/>
       <c r="N110" t="inlineStr"/>
+      <c r="O110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5222,37 +5196,66 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>100</v>
+      </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
-      <c r="I111" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/?curid=40964331</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Tushkings</t>
+        </is>
+      </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="K111" t="inlineStr">
-        <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Kaju+Masala&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
-        </is>
-      </c>
-      <c r="L111" t="inlineStr"/>
-      <c r="M111" t="inlineStr"/>
-      <c r="N111" t="inlineStr"/>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Kaju Masala.jpg</t>
+        </is>
+      </c>
+      <c r="M111" t="n">
+        <v>599735</v>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>1800x1200</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1_JByXVrTLVY3W6diLh_lPkO8Tu24jJ89/view?usp=drivesdk</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5262,7 +5265,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C112" t="inlineStr"/>
@@ -5287,12 +5290,13 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Seekh+Kebab&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/4/47/Chicken_Seekh_Kabab.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
         </is>
       </c>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr"/>
       <c r="N112" t="inlineStr"/>
+      <c r="O112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5327,12 +5331,13 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Veg+KL+Special+Soup&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+          <t>No image candidates found.</t>
         </is>
       </c>
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr"/>
       <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5367,12 +5372,13 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Paneer+Pahadi+Kebab&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Paneer+Pahadi+Kebab+dish&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr"/>
       <c r="N114" t="inlineStr"/>
+      <c r="O114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5413,6 +5419,7 @@
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr"/>
       <c r="N115" t="inlineStr"/>
+      <c r="O115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5453,6 +5460,7 @@
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr"/>
       <c r="N116" t="inlineStr"/>
+      <c r="O116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5493,6 +5501,7 @@
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr"/>
       <c r="N117" t="inlineStr"/>
+      <c r="O117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5533,6 +5542,7 @@
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr"/>
       <c r="N118" t="inlineStr"/>
+      <c r="O118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5573,6 +5583,7 @@
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr"/>
       <c r="N119" t="inlineStr"/>
+      <c r="O119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5613,6 +5624,7 @@
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr"/>
       <c r="N120" t="inlineStr"/>
+      <c r="O120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -5653,6 +5665,7 @@
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr"/>
       <c r="N121" t="inlineStr"/>
+      <c r="O121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -5693,6 +5706,7 @@
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr"/>
       <c r="N122" t="inlineStr"/>
+      <c r="O122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5733,6 +5747,7 @@
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr"/>
       <c r="N123" t="inlineStr"/>
+      <c r="O123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5773,6 +5788,7 @@
       <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr"/>
       <c r="N124" t="inlineStr"/>
+      <c r="O124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5813,6 +5829,7 @@
       <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr"/>
       <c r="N125" t="inlineStr"/>
+      <c r="O125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -5853,6 +5870,7 @@
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr"/>
       <c r="N126" t="inlineStr"/>
+      <c r="O126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -5893,6 +5911,7 @@
       <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr"/>
       <c r="N127" t="inlineStr"/>
+      <c r="O127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -5933,6 +5952,7 @@
       <c r="L128" t="inlineStr"/>
       <c r="M128" t="inlineStr"/>
       <c r="N128" t="inlineStr"/>
+      <c r="O128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -5973,6 +5993,7 @@
       <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr"/>
       <c r="N129" t="inlineStr"/>
+      <c r="O129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6013,6 +6034,7 @@
       <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr"/>
       <c r="N130" t="inlineStr"/>
+      <c r="O130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6053,6 +6075,7 @@
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr"/>
       <c r="N131" t="inlineStr"/>
+      <c r="O131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6093,6 +6116,7 @@
       <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr"/>
       <c r="N132" t="inlineStr"/>
+      <c r="O132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6133,6 +6157,7 @@
       <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr"/>
       <c r="N133" t="inlineStr"/>
+      <c r="O133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -6173,6 +6198,7 @@
       <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr"/>
       <c r="N134" t="inlineStr"/>
+      <c r="O134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -6213,6 +6239,7 @@
       <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr"/>
       <c r="N135" t="inlineStr"/>
+      <c r="O135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -6253,6 +6280,7 @@
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr"/>
       <c r="N136" t="inlineStr"/>
+      <c r="O136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6293,6 +6321,7 @@
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr"/>
       <c r="N137" t="inlineStr"/>
+      <c r="O137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6333,6 +6362,7 @@
       <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr"/>
       <c r="N138" t="inlineStr"/>
+      <c r="O138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6373,6 +6403,7 @@
       <c r="L139" t="inlineStr"/>
       <c r="M139" t="inlineStr"/>
       <c r="N139" t="inlineStr"/>
+      <c r="O139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6413,6 +6444,7 @@
       <c r="L140" t="inlineStr"/>
       <c r="M140" t="inlineStr"/>
       <c r="N140" t="inlineStr"/>
+      <c r="O140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6453,6 +6485,7 @@
       <c r="L141" t="inlineStr"/>
       <c r="M141" t="inlineStr"/>
       <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6493,6 +6526,7 @@
       <c r="L142" t="inlineStr"/>
       <c r="M142" t="inlineStr"/>
       <c r="N142" t="inlineStr"/>
+      <c r="O142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -6502,7 +6536,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C143" t="inlineStr"/>
@@ -6527,12 +6561,13 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/c/ca/Chinese_Dishes_-_Dejavu_-_Meghalaya_-_DSC_005.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Veg+Manchurian+Noodles&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L143" t="inlineStr"/>
       <c r="M143" t="inlineStr"/>
       <c r="N143" t="inlineStr"/>
+      <c r="O143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -6567,12 +6602,13 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>No image candidates found.</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Angara+Kebab&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="inlineStr"/>
       <c r="N144" t="inlineStr"/>
+      <c r="O144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -6582,7 +6618,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C145" t="inlineStr"/>
@@ -6607,12 +6643,13 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/f/f6/Fried_Rice_Chicken_-_Ghin_Khao_%281115240535%29.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Oily+Fry&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr"/>
       <c r="N145" t="inlineStr"/>
+      <c r="O145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -6622,7 +6659,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C146" t="inlineStr"/>
@@ -6647,12 +6684,13 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/f/f4/20251026_Celadon_Ewer_with_Dragon-shaped_Handle_and_Chicken-head_Spout.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
+          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Dragon&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
         </is>
       </c>
       <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr"/>
       <c r="N146" t="inlineStr"/>
+      <c r="O146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -6693,6 +6731,7 @@
       <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr"/>
       <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -6733,6 +6772,7 @@
       <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr"/>
       <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -6773,6 +6813,7 @@
       <c r="L149" t="inlineStr"/>
       <c r="M149" t="inlineStr"/>
       <c r="N149" t="inlineStr"/>
+      <c r="O149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -6813,6 +6854,7 @@
       <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr"/>
       <c r="N150" t="inlineStr"/>
+      <c r="O150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -6853,6 +6895,7 @@
       <c r="L151" t="inlineStr"/>
       <c r="M151" t="inlineStr"/>
       <c r="N151" t="inlineStr"/>
+      <c r="O151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -6893,6 +6936,7 @@
       <c r="L152" t="inlineStr"/>
       <c r="M152" t="inlineStr"/>
       <c r="N152" t="inlineStr"/>
+      <c r="O152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -6933,6 +6977,7 @@
       <c r="L153" t="inlineStr"/>
       <c r="M153" t="inlineStr"/>
       <c r="N153" t="inlineStr"/>
+      <c r="O153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -6973,6 +7018,7 @@
       <c r="L154" t="inlineStr"/>
       <c r="M154" t="inlineStr"/>
       <c r="N154" t="inlineStr"/>
+      <c r="O154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -7013,6 +7059,7 @@
       <c r="L155" t="inlineStr"/>
       <c r="M155" t="inlineStr"/>
       <c r="N155" t="inlineStr"/>
+      <c r="O155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -7053,6 +7100,7 @@
       <c r="L156" t="inlineStr"/>
       <c r="M156" t="inlineStr"/>
       <c r="N156" t="inlineStr"/>
+      <c r="O156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -7093,6 +7141,7 @@
       <c r="L157" t="inlineStr"/>
       <c r="M157" t="inlineStr"/>
       <c r="N157" t="inlineStr"/>
+      <c r="O157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -7133,6 +7182,7 @@
       <c r="L158" t="inlineStr"/>
       <c r="M158" t="inlineStr"/>
       <c r="N158" t="inlineStr"/>
+      <c r="O158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -7173,6 +7223,7 @@
       <c r="L159" t="inlineStr"/>
       <c r="M159" t="inlineStr"/>
       <c r="N159" t="inlineStr"/>
+      <c r="O159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -7213,6 +7264,7 @@
       <c r="L160" t="inlineStr"/>
       <c r="M160" t="inlineStr"/>
       <c r="N160" t="inlineStr"/>
+      <c r="O160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -7253,6 +7305,7 @@
       <c r="L161" t="inlineStr"/>
       <c r="M161" t="inlineStr"/>
       <c r="N161" t="inlineStr"/>
+      <c r="O161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -7293,6 +7346,7 @@
       <c r="L162" t="inlineStr"/>
       <c r="M162" t="inlineStr"/>
       <c r="N162" t="inlineStr"/>
+      <c r="O162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -7333,6 +7387,7 @@
       <c r="L163" t="inlineStr"/>
       <c r="M163" t="inlineStr"/>
       <c r="N163" t="inlineStr"/>
+      <c r="O163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -7373,6 +7428,7 @@
       <c r="L164" t="inlineStr"/>
       <c r="M164" t="inlineStr"/>
       <c r="N164" t="inlineStr"/>
+      <c r="O164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -7413,6 +7469,7 @@
       <c r="L165" t="inlineStr"/>
       <c r="M165" t="inlineStr"/>
       <c r="N165" t="inlineStr"/>
+      <c r="O165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -7422,7 +7479,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
@@ -7447,12 +7504,13 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Afghani&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/1/11/Chicken_2.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
         </is>
       </c>
       <c r="L166" t="inlineStr"/>
       <c r="M166" t="inlineStr"/>
       <c r="N166" t="inlineStr"/>
+      <c r="O166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -7462,7 +7520,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
@@ -7487,12 +7545,13 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Chicken+Tandoor+Masala&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/8/88/Chicken_Tandoor_grilled_in_oven.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
         </is>
       </c>
       <c r="L167" t="inlineStr"/>
       <c r="M167" t="inlineStr"/>
       <c r="N167" t="inlineStr"/>
+      <c r="O167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -7502,37 +7561,66 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>90</v>
+      </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F168" t="inlineStr"/>
-      <c r="G168" t="inlineStr"/>
-      <c r="H168" t="inlineStr"/>
-      <c r="I168" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>https://commons.wikimedia.org/?curid=153312823</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>CC BY-SA 4.0</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Gannu03</t>
+        </is>
+      </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="K168" t="inlineStr">
-        <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Paneer+Masala&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
-        </is>
-      </c>
-      <c r="L168" t="inlineStr"/>
-      <c r="M168" t="inlineStr"/>
-      <c r="N168" t="inlineStr"/>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr"/>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>C:\Users\kusha\Downloads\AI-Food-Image-Agent-Complete\AI-Food-Image-Agent\output\images\Paneer Masala.jpg</t>
+        </is>
+      </c>
+      <c r="M168" t="n">
+        <v>313055</v>
+      </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>1800x1200</t>
+        </is>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/14PDnsBazTDYlgTOf2iZiPC5QYzDZJ4vG/view?usp=drivesdk</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -7542,7 +7630,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C169" t="inlineStr"/>
@@ -7567,12 +7655,13 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>429 Client Error: Too Many Requests for url: https://commons.wikimedia.org/w/api.php?action=query&amp;format=json&amp;generator=search&amp;gsrsearch=Cheesy+Spaghetti&amp;gsrnamespace=6&amp;gsrlimit=5&amp;prop=imageinfo&amp;iiprop=url%7Csize%7Cmime%7Cextmetadata&amp;iiurlwidth=2200</t>
+          <t>429 Client Error: Too many requests - please contact noc@wikimedia.org to discuss a less disruptive approach or instead use thumbnail images in sizes listed on https://w.wiki/GHai. (0c640b1) for url: https://upload.wikimedia.org/wikipedia/commons/0/0a/Spaghetti_in_a_Bowl.jpg?utm_source=commons.wikimedia.org&amp;utm_campaign=imageinfo&amp;utm_content=thumbnail_unscaled</t>
         </is>
       </c>
       <c r="L169" t="inlineStr"/>
       <c r="M169" t="inlineStr"/>
       <c r="N169" t="inlineStr"/>
+      <c r="O169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -7613,6 +7702,7 @@
       <c r="L170" t="inlineStr"/>
       <c r="M170" t="inlineStr"/>
       <c r="N170" t="inlineStr"/>
+      <c r="O170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -7653,6 +7743,7 @@
       <c r="L171" t="inlineStr"/>
       <c r="M171" t="inlineStr"/>
       <c r="N171" t="inlineStr"/>
+      <c r="O171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -7693,6 +7784,7 @@
       <c r="L172" t="inlineStr"/>
       <c r="M172" t="inlineStr"/>
       <c r="N172" t="inlineStr"/>
+      <c r="O172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -7733,6 +7825,7 @@
       <c r="L173" t="inlineStr"/>
       <c r="M173" t="inlineStr"/>
       <c r="N173" t="inlineStr"/>
+      <c r="O173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -7773,6 +7866,7 @@
       <c r="L174" t="inlineStr"/>
       <c r="M174" t="inlineStr"/>
       <c r="N174" t="inlineStr"/>
+      <c r="O174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -7813,6 +7907,7 @@
       <c r="L175" t="inlineStr"/>
       <c r="M175" t="inlineStr"/>
       <c r="N175" t="inlineStr"/>
+      <c r="O175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -7853,6 +7948,7 @@
       <c r="L176" t="inlineStr"/>
       <c r="M176" t="inlineStr"/>
       <c r="N176" t="inlineStr"/>
+      <c r="O176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -7893,6 +7989,7 @@
       <c r="L177" t="inlineStr"/>
       <c r="M177" t="inlineStr"/>
       <c r="N177" t="inlineStr"/>
+      <c r="O177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -7933,6 +8030,7 @@
       <c r="L178" t="inlineStr"/>
       <c r="M178" t="inlineStr"/>
       <c r="N178" t="inlineStr"/>
+      <c r="O178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -7973,6 +8071,7 @@
       <c r="L179" t="inlineStr"/>
       <c r="M179" t="inlineStr"/>
       <c r="N179" t="inlineStr"/>
+      <c r="O179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -8013,6 +8112,7 @@
       <c r="L180" t="inlineStr"/>
       <c r="M180" t="inlineStr"/>
       <c r="N180" t="inlineStr"/>
+      <c r="O180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -8053,6 +8153,7 @@
       <c r="L181" t="inlineStr"/>
       <c r="M181" t="inlineStr"/>
       <c r="N181" t="inlineStr"/>
+      <c r="O181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -8093,6 +8194,7 @@
       <c r="L182" t="inlineStr"/>
       <c r="M182" t="inlineStr"/>
       <c r="N182" t="inlineStr"/>
+      <c r="O182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -8133,6 +8235,7 @@
       <c r="L183" t="inlineStr"/>
       <c r="M183" t="inlineStr"/>
       <c r="N183" t="inlineStr"/>
+      <c r="O183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -8173,6 +8276,7 @@
       <c r="L184" t="inlineStr"/>
       <c r="M184" t="inlineStr"/>
       <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -8213,6 +8317,7 @@
       <c r="L185" t="inlineStr"/>
       <c r="M185" t="inlineStr"/>
       <c r="N185" t="inlineStr"/>
+      <c r="O185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -8253,6 +8358,7 @@
       <c r="L186" t="inlineStr"/>
       <c r="M186" t="inlineStr"/>
       <c r="N186" t="inlineStr"/>
+      <c r="O186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -8293,6 +8399,7 @@
       <c r="L187" t="inlineStr"/>
       <c r="M187" t="inlineStr"/>
       <c r="N187" t="inlineStr"/>
+      <c r="O187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -8333,6 +8440,7 @@
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="inlineStr"/>
       <c r="N188" t="inlineStr"/>
+      <c r="O188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -8373,6 +8481,7 @@
       <c r="L189" t="inlineStr"/>
       <c r="M189" t="inlineStr"/>
       <c r="N189" t="inlineStr"/>
+      <c r="O189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -8413,6 +8522,7 @@
       <c r="L190" t="inlineStr"/>
       <c r="M190" t="inlineStr"/>
       <c r="N190" t="inlineStr"/>
+      <c r="O190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -8453,6 +8563,7 @@
       <c r="L191" t="inlineStr"/>
       <c r="M191" t="inlineStr"/>
       <c r="N191" t="inlineStr"/>
+      <c r="O191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -8493,6 +8604,7 @@
       <c r="L192" t="inlineStr"/>
       <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr"/>
+      <c r="O192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -8533,6 +8645,7 @@
       <c r="L193" t="inlineStr"/>
       <c r="M193" t="inlineStr"/>
       <c r="N193" t="inlineStr"/>
+      <c r="O193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -8573,6 +8686,7 @@
       <c r="L194" t="inlineStr"/>
       <c r="M194" t="inlineStr"/>
       <c r="N194" t="inlineStr"/>
+      <c r="O194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -8613,6 +8727,7 @@
       <c r="L195" t="inlineStr"/>
       <c r="M195" t="inlineStr"/>
       <c r="N195" t="inlineStr"/>
+      <c r="O195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -8653,6 +8768,7 @@
       <c r="L196" t="inlineStr"/>
       <c r="M196" t="inlineStr"/>
       <c r="N196" t="inlineStr"/>
+      <c r="O196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -8693,6 +8809,7 @@
       <c r="L197" t="inlineStr"/>
       <c r="M197" t="inlineStr"/>
       <c r="N197" t="inlineStr"/>
+      <c r="O197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -8733,6 +8850,7 @@
       <c r="L198" t="inlineStr"/>
       <c r="M198" t="inlineStr"/>
       <c r="N198" t="inlineStr"/>
+      <c r="O198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -8773,6 +8891,7 @@
       <c r="L199" t="inlineStr"/>
       <c r="M199" t="inlineStr"/>
       <c r="N199" t="inlineStr"/>
+      <c r="O199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -8813,6 +8932,7 @@
       <c r="L200" t="inlineStr"/>
       <c r="M200" t="inlineStr"/>
       <c r="N200" t="inlineStr"/>
+      <c r="O200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -8853,6 +8973,7 @@
       <c r="L201" t="inlineStr"/>
       <c r="M201" t="inlineStr"/>
       <c r="N201" t="inlineStr"/>
+      <c r="O201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -8893,6 +9014,7 @@
       <c r="L202" t="inlineStr"/>
       <c r="M202" t="inlineStr"/>
       <c r="N202" t="inlineStr"/>
+      <c r="O202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -8933,6 +9055,7 @@
       <c r="L203" t="inlineStr"/>
       <c r="M203" t="inlineStr"/>
       <c r="N203" t="inlineStr"/>
+      <c r="O203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -8973,6 +9096,7 @@
       <c r="L204" t="inlineStr"/>
       <c r="M204" t="inlineStr"/>
       <c r="N204" t="inlineStr"/>
+      <c r="O204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -9013,6 +9137,7 @@
       <c r="L205" t="inlineStr"/>
       <c r="M205" t="inlineStr"/>
       <c r="N205" t="inlineStr"/>
+      <c r="O205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -9053,6 +9178,7 @@
       <c r="L206" t="inlineStr"/>
       <c r="M206" t="inlineStr"/>
       <c r="N206" t="inlineStr"/>
+      <c r="O206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -9093,6 +9219,7 @@
       <c r="L207" t="inlineStr"/>
       <c r="M207" t="inlineStr"/>
       <c r="N207" t="inlineStr"/>
+      <c r="O207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -9133,6 +9260,7 @@
       <c r="L208" t="inlineStr"/>
       <c r="M208" t="inlineStr"/>
       <c r="N208" t="inlineStr"/>
+      <c r="O208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -9173,6 +9301,7 @@
       <c r="L209" t="inlineStr"/>
       <c r="M209" t="inlineStr"/>
       <c r="N209" t="inlineStr"/>
+      <c r="O209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -9213,6 +9342,7 @@
       <c r="L210" t="inlineStr"/>
       <c r="M210" t="inlineStr"/>
       <c r="N210" t="inlineStr"/>
+      <c r="O210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -9253,6 +9383,7 @@
       <c r="L211" t="inlineStr"/>
       <c r="M211" t="inlineStr"/>
       <c r="N211" t="inlineStr"/>
+      <c r="O211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -9293,6 +9424,7 @@
       <c r="L212" t="inlineStr"/>
       <c r="M212" t="inlineStr"/>
       <c r="N212" t="inlineStr"/>
+      <c r="O212" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>